<commit_message>
Add can workbook and adjust will pagination
</commit_message>
<xml_diff>
--- a/Studymaterials/中学生英作文助動詞will編.xlsx
+++ b/Studymaterials/中学生英作文助動詞will編.xlsx
@@ -3732,8 +3732,8 @@
     <mergeCell ref="A81:J81"/>
     <mergeCell ref="A38:J38"/>
     <mergeCell ref="A96:J96"/>
+    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A121:J121"/>
-    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A161:J161"/>
     <mergeCell ref="A13:J13"/>
     <mergeCell ref="A44:J44"/>
@@ -3812,14 +3812,14 @@
     <mergeCell ref="A116:J116"/>
     <mergeCell ref="A85:J85"/>
     <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A131:J131"/>
     <mergeCell ref="A126:J126"/>
-    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A100:J100"/>
     <mergeCell ref="A140:J140"/>
     <mergeCell ref="A53:J53"/>
+    <mergeCell ref="A109:J109"/>
     <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A109:J109"/>
     <mergeCell ref="A129:J129"/>
     <mergeCell ref="A10:J10"/>
     <mergeCell ref="A68:J68"/>
@@ -3857,14 +3857,10 @@
   <printOptions horizontalCentered="1" verticalCentered="1" gridLines="1"/>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1" verticalDpi="0"/>
-  <rowBreaks count="8" manualBreakCount="8">
-    <brk id="20" min="0" max="16383" man="1"/>
+  <rowBreaks count="4" manualBreakCount="4">
     <brk id="38" min="0" max="16383" man="1"/>
-    <brk id="56" min="0" max="16383" man="1"/>
     <brk id="74" min="0" max="16383" man="1"/>
-    <brk id="92" min="0" max="16383" man="1"/>
     <brk id="110" min="0" max="16383" man="1"/>
-    <brk id="128" min="0" max="16383" man="1"/>
     <brk id="146" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
@@ -6531,8 +6527,8 @@
     <mergeCell ref="A81:J81"/>
     <mergeCell ref="A38:J38"/>
     <mergeCell ref="A96:J96"/>
+    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A121:J121"/>
-    <mergeCell ref="A147:J147"/>
     <mergeCell ref="A161:J161"/>
     <mergeCell ref="A13:J13"/>
     <mergeCell ref="A44:J44"/>
@@ -6611,14 +6607,14 @@
     <mergeCell ref="A116:J116"/>
     <mergeCell ref="A85:J85"/>
     <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A131:J131"/>
     <mergeCell ref="A126:J126"/>
-    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A100:J100"/>
     <mergeCell ref="A140:J140"/>
     <mergeCell ref="A53:J53"/>
+    <mergeCell ref="A109:J109"/>
     <mergeCell ref="A35:J35"/>
-    <mergeCell ref="A109:J109"/>
     <mergeCell ref="A129:J129"/>
     <mergeCell ref="A10:J10"/>
     <mergeCell ref="A68:J68"/>
@@ -6656,14 +6652,10 @@
   <printOptions horizontalCentered="1" verticalCentered="1" gridLines="1"/>
   <pageMargins left="0.45" right="0.45" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1" verticalDpi="0"/>
-  <rowBreaks count="8" manualBreakCount="8">
-    <brk id="20" min="0" max="16383" man="1"/>
+  <rowBreaks count="4" manualBreakCount="4">
     <brk id="38" min="0" max="16383" man="1"/>
-    <brk id="56" min="0" max="16383" man="1"/>
     <brk id="74" min="0" max="16383" man="1"/>
-    <brk id="92" min="0" max="16383" man="1"/>
     <brk id="110" min="0" max="16383" man="1"/>
-    <brk id="128" min="0" max="16383" man="1"/>
     <brk id="146" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>

</xml_diff>